<commit_message>
update planning after implementation phase 1
</commit_message>
<xml_diff>
--- a/organisation/Zeitplan.xlsx
+++ b/organisation/Zeitplan.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\Vincent\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vince\Downloads\M306-Projektarbeit\organisation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00315A8B-7D23-449D-BE48-6EA8CC78646F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10DC720A-D918-4D86-B879-2579A7C2545C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Zeitplan" sheetId="1" r:id="rId1"/>
@@ -380,18 +380,18 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="1" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -707,10 +707,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:19" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="19" t="s">
         <v>67</v>
       </c>
-      <c r="B1" s="19"/>
+      <c r="B1" s="20"/>
       <c r="C1" s="2">
         <v>46146</v>
       </c>
@@ -726,42 +726,42 @@
       <c r="C3" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="15">
+      <c r="D3" s="17">
         <f>$C$1+0*7</f>
         <v>46146</v>
       </c>
       <c r="E3" s="16"/>
-      <c r="F3" s="15">
+      <c r="F3" s="17">
         <f>$C$1+1*7</f>
         <v>46153</v>
       </c>
       <c r="G3" s="16"/>
-      <c r="H3" s="15">
+      <c r="H3" s="17">
         <f>$C$1+2*7</f>
         <v>46160</v>
       </c>
       <c r="I3" s="16"/>
-      <c r="J3" s="15">
+      <c r="J3" s="17">
         <f>$C$1+3*7</f>
         <v>46167</v>
       </c>
       <c r="K3" s="16"/>
-      <c r="L3" s="15">
+      <c r="L3" s="17">
         <f>$C$1+4*7</f>
         <v>46174</v>
       </c>
       <c r="M3" s="16"/>
-      <c r="N3" s="15">
+      <c r="N3" s="17">
         <f>$C$1+5*7</f>
         <v>46181</v>
       </c>
       <c r="O3" s="16"/>
-      <c r="P3" s="15">
+      <c r="P3" s="17">
         <f>$C$1+6*7</f>
         <v>46188</v>
       </c>
       <c r="Q3" s="16"/>
-      <c r="R3" s="15">
+      <c r="R3" s="17">
         <f>$C$1+7*7</f>
         <v>46195</v>
       </c>
@@ -821,7 +821,7 @@
       </c>
     </row>
     <row r="5" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="17" t="s">
+      <c r="A5" s="15" t="s">
         <v>5</v>
       </c>
       <c r="B5" s="10" t="s">
@@ -948,7 +948,7 @@
       <c r="S9" s="7"/>
     </row>
     <row r="10" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="17" t="s">
+      <c r="A10" s="15" t="s">
         <v>16</v>
       </c>
       <c r="B10" s="10" t="s">
@@ -961,7 +961,7 @@
       <c r="E10" s="7"/>
       <c r="F10" s="7"/>
       <c r="G10" s="7"/>
-      <c r="H10" s="13"/>
+      <c r="H10" s="12"/>
       <c r="I10" s="7"/>
       <c r="J10" s="7"/>
       <c r="K10" s="7"/>
@@ -986,7 +986,7 @@
       <c r="E11" s="7"/>
       <c r="F11" s="7"/>
       <c r="G11" s="7"/>
-      <c r="H11" s="13"/>
+      <c r="H11" s="12"/>
       <c r="I11" s="7"/>
       <c r="J11" s="7"/>
       <c r="K11" s="7"/>
@@ -1012,7 +1012,7 @@
       <c r="F12" s="7"/>
       <c r="G12" s="7"/>
       <c r="H12" s="7"/>
-      <c r="I12" s="13"/>
+      <c r="I12" s="12"/>
       <c r="J12" s="7"/>
       <c r="K12" s="7"/>
       <c r="L12" s="7"/>
@@ -1039,7 +1039,7 @@
       <c r="F13" s="7"/>
       <c r="G13" s="7"/>
       <c r="H13" s="7"/>
-      <c r="I13" s="13"/>
+      <c r="I13" s="12"/>
       <c r="J13" s="7"/>
       <c r="K13" s="7"/>
       <c r="L13" s="7"/>
@@ -1052,7 +1052,7 @@
       <c r="S13" s="7"/>
     </row>
     <row r="14" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="17" t="s">
+      <c r="A14" s="15" t="s">
         <v>26</v>
       </c>
       <c r="B14" s="10" t="s">
@@ -1067,7 +1067,7 @@
       <c r="G14" s="7"/>
       <c r="H14" s="7"/>
       <c r="I14" s="7"/>
-      <c r="J14" s="13"/>
+      <c r="J14" s="12"/>
       <c r="K14" s="7"/>
       <c r="L14" s="7"/>
       <c r="M14" s="7"/>
@@ -1090,7 +1090,7 @@
       <c r="G15" s="7"/>
       <c r="H15" s="7"/>
       <c r="I15" s="7"/>
-      <c r="J15" s="13"/>
+      <c r="J15" s="12"/>
       <c r="K15" s="7"/>
       <c r="L15" s="7"/>
       <c r="M15" s="7"/>
@@ -1114,7 +1114,7 @@
       <c r="H16" s="7"/>
       <c r="I16" s="7"/>
       <c r="J16" s="7"/>
-      <c r="K16" s="13"/>
+      <c r="K16" s="12"/>
       <c r="L16" s="7"/>
       <c r="M16" s="7"/>
       <c r="N16" s="7"/>
@@ -1138,7 +1138,7 @@
       <c r="I17" s="7"/>
       <c r="J17" s="7"/>
       <c r="K17" s="7"/>
-      <c r="L17" s="13"/>
+      <c r="L17" s="12"/>
       <c r="M17" s="7"/>
       <c r="N17" s="7"/>
       <c r="O17" s="7"/>
@@ -1162,7 +1162,7 @@
       <c r="J18" s="7"/>
       <c r="K18" s="7"/>
       <c r="L18" s="7"/>
-      <c r="M18" s="13"/>
+      <c r="M18" s="12"/>
       <c r="N18" s="7"/>
       <c r="O18" s="7"/>
       <c r="P18" s="7"/>
@@ -1217,7 +1217,7 @@
       <c r="S20" s="7"/>
     </row>
     <row r="21" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="17" t="s">
+      <c r="A21" s="15" t="s">
         <v>35</v>
       </c>
       <c r="B21" s="10" t="s">
@@ -1269,7 +1269,7 @@
       <c r="S22" s="7"/>
     </row>
     <row r="23" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="17" t="s">
+      <c r="A23" s="15" t="s">
         <v>40</v>
       </c>
       <c r="B23" s="10" t="s">
@@ -1421,7 +1421,7 @@
       <c r="S28" s="7"/>
     </row>
     <row r="29" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="17" t="s">
+      <c r="A29" s="15" t="s">
         <v>53</v>
       </c>
       <c r="B29" s="10" t="s">
@@ -1434,12 +1434,12 @@
       <c r="E29" s="12"/>
       <c r="F29" s="12"/>
       <c r="G29" s="12"/>
-      <c r="H29" s="13"/>
-      <c r="I29" s="13"/>
-      <c r="J29" s="13"/>
-      <c r="K29" s="13"/>
-      <c r="L29" s="13"/>
-      <c r="M29" s="13"/>
+      <c r="H29" s="12"/>
+      <c r="I29" s="12"/>
+      <c r="J29" s="12"/>
+      <c r="K29" s="12"/>
+      <c r="L29" s="12"/>
+      <c r="M29" s="12"/>
       <c r="N29" s="13"/>
       <c r="O29" s="13"/>
       <c r="P29" s="13"/>
@@ -1460,11 +1460,11 @@
       <c r="F30" s="7"/>
       <c r="G30" s="12"/>
       <c r="H30" s="7"/>
-      <c r="I30" s="13"/>
+      <c r="I30" s="12"/>
       <c r="J30" s="7"/>
-      <c r="K30" s="13"/>
+      <c r="K30" s="12"/>
       <c r="L30" s="7"/>
-      <c r="M30" s="13"/>
+      <c r="M30" s="12"/>
       <c r="N30" s="7"/>
       <c r="O30" s="13"/>
       <c r="P30" s="7"/>
@@ -1473,7 +1473,7 @@
       <c r="S30" s="13"/>
     </row>
     <row r="31" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="17" t="s">
+      <c r="A31" s="15" t="s">
         <v>58</v>
       </c>
       <c r="B31" s="10" t="s">

</xml_diff>

<commit_message>
updated documentation to be more requirement compliant
</commit_message>
<xml_diff>
--- a/organisation/Zeitplan.xlsx
+++ b/organisation/Zeitplan.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vince\Downloads\M306-Projektarbeit\organisation\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alex\source\repos\M306-Projektarbeit\organisation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10DC720A-D918-4D86-B879-2579A7C2545C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E436E08-5FCA-4409-8932-9AB1D06709F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="27634" windowHeight="14914" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Zeitplan" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="74">
   <si>
     <t>Phase</t>
   </si>
@@ -240,6 +240,24 @@
   </si>
   <si>
     <t>Startdatum:</t>
+  </si>
+  <si>
+    <t>Aufsetzen Repository/Libraries</t>
+  </si>
+  <si>
+    <t>Arbeit Globus</t>
+  </si>
+  <si>
+    <t>Projektionen auf Globus</t>
+  </si>
+  <si>
+    <t>API Fetching/Filtering</t>
+  </si>
+  <si>
+    <t>API verarbeitbar für globus</t>
+  </si>
+  <si>
+    <t>Integration satelliten + globus</t>
   </si>
 </sst>
 </file>
@@ -380,18 +398,18 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="164" fontId="1" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="164" fontId="1" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -698,7 +716,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:S37"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="6" customWidth="1"/>
@@ -706,71 +724,71 @@
     <col min="4" max="19" width="7" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="19" t="s">
+    <row r="1" spans="1:19" ht="22" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A1" s="15" t="s">
         <v>67</v>
       </c>
-      <c r="B1" s="20"/>
+      <c r="B1" s="16"/>
       <c r="C1" s="2">
         <v>46146</v>
       </c>
     </row>
-    <row r="2" spans="1:19" ht="8.1" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="3" spans="1:19" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="18" t="s">
+    <row r="2" spans="1:19" ht="8.15" customHeight="1" x14ac:dyDescent="0.4"/>
+    <row r="3" spans="1:19" ht="22" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A3" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="18" t="s">
+      <c r="B3" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="18" t="s">
+      <c r="C3" s="20" t="s">
         <v>2</v>
       </c>
       <c r="D3" s="17">
         <f>$C$1+0*7</f>
         <v>46146</v>
       </c>
-      <c r="E3" s="16"/>
+      <c r="E3" s="18"/>
       <c r="F3" s="17">
         <f>$C$1+1*7</f>
         <v>46153</v>
       </c>
-      <c r="G3" s="16"/>
+      <c r="G3" s="18"/>
       <c r="H3" s="17">
         <f>$C$1+2*7</f>
         <v>46160</v>
       </c>
-      <c r="I3" s="16"/>
+      <c r="I3" s="18"/>
       <c r="J3" s="17">
         <f>$C$1+3*7</f>
         <v>46167</v>
       </c>
-      <c r="K3" s="16"/>
+      <c r="K3" s="18"/>
       <c r="L3" s="17">
         <f>$C$1+4*7</f>
         <v>46174</v>
       </c>
-      <c r="M3" s="16"/>
+      <c r="M3" s="18"/>
       <c r="N3" s="17">
         <f>$C$1+5*7</f>
         <v>46181</v>
       </c>
-      <c r="O3" s="16"/>
+      <c r="O3" s="18"/>
       <c r="P3" s="17">
         <f>$C$1+6*7</f>
         <v>46188</v>
       </c>
-      <c r="Q3" s="16"/>
+      <c r="Q3" s="18"/>
       <c r="R3" s="17">
         <f>$C$1+7*7</f>
         <v>46195</v>
       </c>
-      <c r="S3" s="16"/>
-    </row>
-    <row r="4" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="16"/>
-      <c r="B4" s="16"/>
-      <c r="C4" s="16"/>
+      <c r="S3" s="18"/>
+    </row>
+    <row r="4" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A4" s="18"/>
+      <c r="B4" s="18"/>
+      <c r="C4" s="18"/>
       <c r="D4" s="8" t="s">
         <v>3</v>
       </c>
@@ -820,8 +838,8 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="15" t="s">
+    <row r="5" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A5" s="19" t="s">
         <v>5</v>
       </c>
       <c r="B5" s="10" t="s">
@@ -847,8 +865,8 @@
       <c r="R5" s="7"/>
       <c r="S5" s="7"/>
     </row>
-    <row r="6" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="16"/>
+    <row r="6" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A6" s="18"/>
       <c r="B6" s="10" t="s">
         <v>8</v>
       </c>
@@ -872,8 +890,8 @@
       <c r="R6" s="7"/>
       <c r="S6" s="7"/>
     </row>
-    <row r="7" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="16"/>
+    <row r="7" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A7" s="18"/>
       <c r="B7" s="10" t="s">
         <v>10</v>
       </c>
@@ -897,8 +915,8 @@
       <c r="R7" s="7"/>
       <c r="S7" s="7"/>
     </row>
-    <row r="8" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="16"/>
+    <row r="8" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A8" s="18"/>
       <c r="B8" s="10" t="s">
         <v>12</v>
       </c>
@@ -922,8 +940,8 @@
       <c r="R8" s="7"/>
       <c r="S8" s="7"/>
     </row>
-    <row r="9" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="16"/>
+    <row r="9" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A9" s="18"/>
       <c r="B9" s="10" t="s">
         <v>14</v>
       </c>
@@ -947,8 +965,8 @@
       <c r="R9" s="7"/>
       <c r="S9" s="7"/>
     </row>
-    <row r="10" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="15" t="s">
+    <row r="10" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A10" s="19" t="s">
         <v>16</v>
       </c>
       <c r="B10" s="10" t="s">
@@ -974,8 +992,8 @@
       <c r="R10" s="7"/>
       <c r="S10" s="7"/>
     </row>
-    <row r="11" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="16"/>
+    <row r="11" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A11" s="18"/>
       <c r="B11" s="10" t="s">
         <v>19</v>
       </c>
@@ -999,8 +1017,8 @@
       <c r="R11" s="7"/>
       <c r="S11" s="7"/>
     </row>
-    <row r="12" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="16"/>
+    <row r="12" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A12" s="18"/>
       <c r="B12" s="10" t="s">
         <v>21</v>
       </c>
@@ -1024,7 +1042,7 @@
       <c r="R12" s="7"/>
       <c r="S12" s="7"/>
     </row>
-    <row r="13" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A13" s="9" t="s">
         <v>23</v>
       </c>
@@ -1051,8 +1069,8 @@
       <c r="R13" s="7"/>
       <c r="S13" s="7"/>
     </row>
-    <row r="14" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="15" t="s">
+    <row r="14" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A14" s="19" t="s">
         <v>26</v>
       </c>
       <c r="B14" s="10" t="s">
@@ -1078,12 +1096,14 @@
       <c r="R14" s="7"/>
       <c r="S14" s="7"/>
     </row>
-    <row r="15" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="16"/>
+    <row r="15" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A15" s="18"/>
       <c r="B15" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="C15" s="11"/>
+      <c r="C15" s="11" t="s">
+        <v>68</v>
+      </c>
       <c r="D15" s="7"/>
       <c r="E15" s="7"/>
       <c r="F15" s="7"/>
@@ -1101,12 +1121,14 @@
       <c r="R15" s="7"/>
       <c r="S15" s="7"/>
     </row>
-    <row r="16" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="16"/>
+    <row r="16" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A16" s="18"/>
       <c r="B16" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="C16" s="11"/>
+      <c r="C16" s="11" t="s">
+        <v>69</v>
+      </c>
       <c r="D16" s="7"/>
       <c r="E16" s="7"/>
       <c r="F16" s="7"/>
@@ -1124,12 +1146,14 @@
       <c r="R16" s="7"/>
       <c r="S16" s="7"/>
     </row>
-    <row r="17" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="16"/>
+    <row r="17" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A17" s="18"/>
       <c r="B17" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="C17" s="11"/>
+      <c r="C17" s="11" t="s">
+        <v>70</v>
+      </c>
       <c r="D17" s="7"/>
       <c r="E17" s="7"/>
       <c r="F17" s="7"/>
@@ -1139,7 +1163,7 @@
       <c r="J17" s="7"/>
       <c r="K17" s="7"/>
       <c r="L17" s="12"/>
-      <c r="M17" s="7"/>
+      <c r="M17" s="3"/>
       <c r="N17" s="7"/>
       <c r="O17" s="7"/>
       <c r="P17" s="7"/>
@@ -1147,12 +1171,14 @@
       <c r="R17" s="7"/>
       <c r="S17" s="7"/>
     </row>
-    <row r="18" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="16"/>
+    <row r="18" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A18" s="18"/>
       <c r="B18" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="C18" s="11"/>
+      <c r="C18" s="11" t="s">
+        <v>71</v>
+      </c>
       <c r="D18" s="7"/>
       <c r="E18" s="7"/>
       <c r="F18" s="7"/>
@@ -1170,12 +1196,14 @@
       <c r="R18" s="7"/>
       <c r="S18" s="7"/>
     </row>
-    <row r="19" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="16"/>
+    <row r="19" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A19" s="18"/>
       <c r="B19" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="C19" s="11"/>
+      <c r="C19" s="11" t="s">
+        <v>72</v>
+      </c>
       <c r="D19" s="7"/>
       <c r="E19" s="7"/>
       <c r="F19" s="7"/>
@@ -1193,12 +1221,14 @@
       <c r="R19" s="7"/>
       <c r="S19" s="7"/>
     </row>
-    <row r="20" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="16"/>
+    <row r="20" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A20" s="18"/>
       <c r="B20" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="C20" s="11"/>
+      <c r="C20" s="11" t="s">
+        <v>73</v>
+      </c>
       <c r="D20" s="7"/>
       <c r="E20" s="7"/>
       <c r="F20" s="7"/>
@@ -1216,8 +1246,8 @@
       <c r="R20" s="7"/>
       <c r="S20" s="7"/>
     </row>
-    <row r="21" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="15" t="s">
+    <row r="21" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A21" s="19" t="s">
         <v>35</v>
       </c>
       <c r="B21" s="10" t="s">
@@ -1243,8 +1273,8 @@
       <c r="R21" s="7"/>
       <c r="S21" s="7"/>
     </row>
-    <row r="22" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="16"/>
+    <row r="22" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A22" s="18"/>
       <c r="B22" s="10" t="s">
         <v>38</v>
       </c>
@@ -1268,8 +1298,8 @@
       <c r="R22" s="7"/>
       <c r="S22" s="7"/>
     </row>
-    <row r="23" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="15" t="s">
+    <row r="23" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A23" s="19" t="s">
         <v>40</v>
       </c>
       <c r="B23" s="10" t="s">
@@ -1295,8 +1325,8 @@
       <c r="R23" s="7"/>
       <c r="S23" s="7"/>
     </row>
-    <row r="24" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="16"/>
+    <row r="24" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A24" s="18"/>
       <c r="B24" s="10" t="s">
         <v>43</v>
       </c>
@@ -1320,8 +1350,8 @@
       <c r="R24" s="7"/>
       <c r="S24" s="7"/>
     </row>
-    <row r="25" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="16"/>
+    <row r="25" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A25" s="18"/>
       <c r="B25" s="10" t="s">
         <v>45</v>
       </c>
@@ -1345,8 +1375,8 @@
       <c r="R25" s="7"/>
       <c r="S25" s="7"/>
     </row>
-    <row r="26" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="16"/>
+    <row r="26" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A26" s="18"/>
       <c r="B26" s="10" t="s">
         <v>47</v>
       </c>
@@ -1370,8 +1400,8 @@
       <c r="R26" s="13"/>
       <c r="S26" s="7"/>
     </row>
-    <row r="27" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="16"/>
+    <row r="27" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A27" s="18"/>
       <c r="B27" s="10" t="s">
         <v>49</v>
       </c>
@@ -1395,8 +1425,8 @@
       <c r="R27" s="13"/>
       <c r="S27" s="7"/>
     </row>
-    <row r="28" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="16"/>
+    <row r="28" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A28" s="18"/>
       <c r="B28" s="10" t="s">
         <v>51</v>
       </c>
@@ -1420,8 +1450,8 @@
       <c r="R28" s="13"/>
       <c r="S28" s="7"/>
     </row>
-    <row r="29" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="15" t="s">
+    <row r="29" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A29" s="19" t="s">
         <v>53</v>
       </c>
       <c r="B29" s="10" t="s">
@@ -1447,8 +1477,8 @@
       <c r="R29" s="13"/>
       <c r="S29" s="13"/>
     </row>
-    <row r="30" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="16"/>
+    <row r="30" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A30" s="18"/>
       <c r="B30" s="10" t="s">
         <v>56</v>
       </c>
@@ -1472,8 +1502,8 @@
       <c r="R30" s="7"/>
       <c r="S30" s="13"/>
     </row>
-    <row r="31" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="15" t="s">
+    <row r="31" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A31" s="19" t="s">
         <v>58</v>
       </c>
       <c r="B31" s="10" t="s">
@@ -1499,8 +1529,8 @@
       <c r="R31" s="7"/>
       <c r="S31" s="14"/>
     </row>
-    <row r="32" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="16"/>
+    <row r="32" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A32" s="18"/>
       <c r="B32" s="10" t="s">
         <v>61</v>
       </c>
@@ -1524,24 +1554,24 @@
       <c r="R32" s="7"/>
       <c r="S32" s="13"/>
     </row>
-    <row r="34" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:3" x14ac:dyDescent="0.4">
       <c r="B34" s="1" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="35" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:3" x14ac:dyDescent="0.4">
       <c r="B35" s="4"/>
       <c r="C35" s="6" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="36" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:3" x14ac:dyDescent="0.4">
       <c r="B36" s="3"/>
       <c r="C36" s="6" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="37" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:3" x14ac:dyDescent="0.4">
       <c r="B37" s="5"/>
       <c r="C37" s="6" t="s">
         <v>66</v>
@@ -1549,11 +1579,6 @@
     </row>
   </sheetData>
   <mergeCells count="19">
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="L3:M3"/>
-    <mergeCell ref="A14:A20"/>
-    <mergeCell ref="A21:A22"/>
     <mergeCell ref="A29:A30"/>
     <mergeCell ref="A31:A32"/>
     <mergeCell ref="R3:S3"/>
@@ -1568,6 +1593,11 @@
     <mergeCell ref="A10:A12"/>
     <mergeCell ref="A5:A9"/>
     <mergeCell ref="B3:B4"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="L3:M3"/>
+    <mergeCell ref="A14:A20"/>
+    <mergeCell ref="A21:A22"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" fitToHeight="0" orientation="landscape"/>

</xml_diff>